<commit_message>
2NF - Abiem Mahmud
</commit_message>
<xml_diff>
--- a/Normalisasi_SalesDB_Abiem Mahmud.xlsx
+++ b/Normalisasi_SalesDB_Abiem Mahmud.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arjia\magang\Latihan-database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49839E2F-4833-4113-827A-AE38C7FE0DDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80CCB380-77BB-4E7E-9502-67D861BF0B1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Petunjuk" sheetId="1" r:id="rId1"/>
@@ -85,8 +85,46 @@
 </comments>
 </file>
 
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Trainer</author>
+  </authors>
+  <commentList>
+    <comment ref="M12" authorId="0" shapeId="0" xr:uid="{0E34D2CD-C0BB-4108-B806-3F26DF3D34F1}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Nilai tertulis di faktur asli (data sumber). Nilai ini dipertahankan sampai 3NF, lalu di sheet 4_3NF dibuktikan bahwa nilainya bisa dihitung ulang dari Qty × Harga.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M13" authorId="0" shapeId="0" xr:uid="{48FA22C1-F622-45F5-B3ED-82588A00B440}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Nilai tertulis di faktur asli (data sumber). Nilai ini dipertahankan sampai 3NF, lalu di sheet 4_3NF dibuktikan bahwa nilainya bisa dihitung ulang dari Qty × Harga.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="156">
   <si>
     <t>Latihan Normalisasi SalesDB — dari data faktur (UNF) sampai 3NF</t>
   </si>
@@ -507,6 +545,87 @@
   </si>
   <si>
     <t>no faktur -&gt; tanggal; kode pelanggan -&gt; nama pelanggan, email, kota; kode produk -&gt; nama produk, harga satuan; kode kategori -&gt; nama kategori</t>
+  </si>
+  <si>
+    <t>tanggal</t>
+  </si>
+  <si>
+    <t>nama pelanggan</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>kota</t>
+  </si>
+  <si>
+    <t>nama</t>
+  </si>
+  <si>
+    <t>harga</t>
+  </si>
+  <si>
+    <t>nama kategori</t>
+  </si>
+  <si>
+    <t>nofaktur, kode pelanggan, kode porduk, kode kategori</t>
+  </si>
+  <si>
+    <t>no faktur (PK)</t>
+  </si>
+  <si>
+    <t>kode pelanggan (FK)</t>
+  </si>
+  <si>
+    <t>faktur</t>
+  </si>
+  <si>
+    <t>qty</t>
+  </si>
+  <si>
+    <t>kode pelanggan (PK)</t>
+  </si>
+  <si>
+    <t>kode produk (PK)</t>
+  </si>
+  <si>
+    <t>k01</t>
+  </si>
+  <si>
+    <t>k03</t>
+  </si>
+  <si>
+    <t>k02</t>
+  </si>
+  <si>
+    <t>kode kategori (FK)</t>
+  </si>
+  <si>
+    <t>kode kategori (PK)</t>
+  </si>
+  <si>
+    <t>no faktur (FK)</t>
+  </si>
+  <si>
+    <t>kode produk (FK)</t>
+  </si>
+  <si>
+    <t>pelanggan</t>
+  </si>
+  <si>
+    <t>produk</t>
+  </si>
+  <si>
+    <t>kategori</t>
+  </si>
+  <si>
+    <t>no faktur -&gt; tanggal; kode pelanggan -&gt; nama pelanggan, email, kota; kode produk -&gt; nama produk, harga satuan; kode kategori -&gt; nama kategori; nofaktur &amp; kode produk -&gt; qty</t>
+  </si>
+  <si>
+    <t>Memisahkan data berdasarkan dependencynya</t>
+  </si>
+  <si>
+    <t>detail faktur</t>
   </si>
 </sst>
 </file>
@@ -516,7 +635,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -569,8 +688,20 @@
       <sz val="10"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -602,8 +733,20 @@
         <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -626,11 +769,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -663,6 +817,42 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1465,8 +1655,8 @@
   <dimension ref="A1:M23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="36.5546875" customWidth="1"/>
-    <col min="2" max="2" width="129" customWidth="1"/>
+    <col min="1" max="1" width="19.109375" customWidth="1"/>
+    <col min="2" max="2" width="30.77734375" customWidth="1"/>
     <col min="3" max="3" width="12.77734375" customWidth="1"/>
     <col min="4" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="24.33203125" customWidth="1"/>
@@ -2068,69 +2258,1133 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:T38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="13" width="19" customWidth="1"/>
+    <col min="14" max="14" width="16.6640625" customWidth="1"/>
+    <col min="15" max="15" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="16"/>
+      <c r="B6" s="16" t="s">
+        <v>136</v>
+      </c>
       <c r="C6" s="17" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="16"/>
+      <c r="B7" s="16" t="s">
+        <v>153</v>
+      </c>
       <c r="C7" s="17" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="16"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B8" s="16" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="18"/>
+    <row r="11" spans="1:13" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="J11" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="L11" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="M11" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="13">
+        <v>46266</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="I12" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="J12" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K12" s="12">
+        <v>1</v>
+      </c>
+      <c r="L12" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="M12" s="14">
+        <v>2150000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="13">
+        <v>46266</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="I13" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="J13" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="K13" s="12">
+        <v>2</v>
+      </c>
+      <c r="L13" s="12">
+        <v>150</v>
+      </c>
+      <c r="M13" s="14">
+        <v>2150000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="13">
+        <v>46275</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="I14" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="J14" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="K14" s="12">
+        <v>1</v>
+      </c>
+      <c r="L14" s="12">
+        <v>750</v>
+      </c>
+      <c r="M14" s="14">
+        <v>900000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="13">
+        <v>46275</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="I15" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="J15" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="K15" s="12">
+        <v>1</v>
+      </c>
+      <c r="L15" s="12">
+        <v>150</v>
+      </c>
+      <c r="M15" s="14">
+        <v>900000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="13">
+        <v>46277</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="I16" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="J16" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K16" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="L16" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="M16" s="14">
+        <v>1050000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A17" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17" s="13">
+        <v>46280</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="J17" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="K17" s="12">
+        <v>10</v>
+      </c>
+      <c r="L17" s="12">
+        <v>25</v>
+      </c>
+      <c r="M17" s="14">
+        <v>346000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="13">
+        <v>46280</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="I18" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="J18" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="K18" s="12">
+        <v>2</v>
+      </c>
+      <c r="L18" s="12">
+        <v>48</v>
+      </c>
+      <c r="M18" s="14">
+        <v>346000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="13">
+        <v>46283</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="J19" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K19" s="12">
+        <v>1</v>
+      </c>
+      <c r="L19" s="12">
+        <v>375</v>
+      </c>
+      <c r="M19" s="14">
+        <v>548000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A20" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" s="13">
+        <v>46283</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="H20" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="I20" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="K20" s="12">
+        <v>5</v>
+      </c>
+      <c r="L20" s="12">
+        <v>25</v>
+      </c>
+      <c r="M20" s="14">
+        <v>548000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B21" s="13">
+        <v>46283</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="H21" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="I21" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="J21" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="K21" s="12">
+        <v>1</v>
+      </c>
+      <c r="L21" s="12">
+        <v>48</v>
+      </c>
+      <c r="M21" s="14">
+        <v>548000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="13">
+        <v>46285</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="I22" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K22" s="12">
+        <v>2</v>
+      </c>
+      <c r="L22" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="M22" s="14">
+        <v>4450000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" s="13">
+        <v>46285</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="H23" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="I23" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="J23" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="K23" s="12">
+        <v>1</v>
+      </c>
+      <c r="L23" s="12">
+        <v>750</v>
+      </c>
+      <c r="M23" s="14">
+        <v>4450000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>139</v>
+      </c>
+      <c r="E25" s="21" t="s">
+        <v>150</v>
+      </c>
+      <c r="J25" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="O25" t="s">
+        <v>152</v>
+      </c>
+      <c r="R25" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" s="25" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A26" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="B26" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="D26" s="24"/>
+      <c r="E26" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="F26" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="G26" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="H26" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="I26" s="24"/>
+      <c r="J26" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="K26" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="L26" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="M26" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="N26" s="24"/>
+      <c r="O26" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="P26" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="Q26" s="32"/>
+      <c r="R26" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="S26" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="T26" s="22" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" s="30" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B27" s="27">
+        <v>46266</v>
+      </c>
+      <c r="C27" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="D27" s="28"/>
+      <c r="E27" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="F27" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="G27" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="H27" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="I27" s="28"/>
+      <c r="J27" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="K27" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="L27" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="M27" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="N27" s="28"/>
+      <c r="O27" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="P27" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q27" s="28"/>
+      <c r="R27" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="S27" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="T27" s="26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" s="30" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" s="27">
+        <v>46275</v>
+      </c>
+      <c r="C28" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" s="28"/>
+      <c r="E28" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="F28" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="G28" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="H28" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="I28" s="28"/>
+      <c r="J28" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="K28" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="L28" s="26">
+        <v>150</v>
+      </c>
+      <c r="M28" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="N28" s="28"/>
+      <c r="O28" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="P28" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q28" s="28"/>
+      <c r="R28" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="S28" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="T28" s="26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" s="30" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" s="27">
+        <v>46277</v>
+      </c>
+      <c r="C29" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="D29" s="28"/>
+      <c r="E29" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="F29" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="G29" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="H29" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="I29" s="28"/>
+      <c r="J29" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="K29" s="26" t="s">
+        <v>119</v>
+      </c>
+      <c r="L29" s="26">
+        <v>750</v>
+      </c>
+      <c r="M29" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="N29" s="28"/>
+      <c r="O29" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="P29" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="Q29" s="28"/>
+      <c r="R29" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="S29" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="T29" s="26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="B30" s="27">
+        <v>46280</v>
+      </c>
+      <c r="C30" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="K30" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="L30" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="M30" s="31" t="s">
+        <v>143</v>
+      </c>
+      <c r="N30" s="28"/>
+      <c r="O30" s="28"/>
+      <c r="P30" s="28"/>
+      <c r="Q30" s="28"/>
+      <c r="R30" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="S30" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="T30" s="26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="B31" s="27">
+        <v>46283</v>
+      </c>
+      <c r="C31" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="D31" s="28"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="26"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="26"/>
+      <c r="I31" s="28"/>
+      <c r="J31" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="K31" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="L31" s="26">
+        <v>25</v>
+      </c>
+      <c r="M31" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="N31" s="28"/>
+      <c r="O31" s="26"/>
+      <c r="P31" s="26"/>
+      <c r="Q31" s="28"/>
+      <c r="R31" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="S31" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="T31" s="26" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" s="27">
+        <v>46285</v>
+      </c>
+      <c r="C32" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="D32" s="28"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="26"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="26"/>
+      <c r="I32" s="28"/>
+      <c r="J32" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="K32" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="L32" s="26">
+        <v>48</v>
+      </c>
+      <c r="M32" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="N32" s="28"/>
+      <c r="O32" s="26"/>
+      <c r="P32" s="26"/>
+      <c r="Q32" s="28"/>
+      <c r="R32" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="S32" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="T32" s="26">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D33" s="28"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="26"/>
+      <c r="G33" s="26"/>
+      <c r="H33" s="26"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="26"/>
+      <c r="K33" s="26"/>
+      <c r="L33" s="26"/>
+      <c r="M33" s="28"/>
+      <c r="N33" s="28"/>
+      <c r="O33" s="28"/>
+      <c r="P33" s="28"/>
+      <c r="Q33" s="28"/>
+      <c r="R33" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="S33" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="T33" s="26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="26"/>
+      <c r="B34" s="27"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="26"/>
+      <c r="F34" s="26"/>
+      <c r="G34" s="26"/>
+      <c r="H34" s="26"/>
+      <c r="I34" s="28"/>
+      <c r="J34" s="26"/>
+      <c r="K34" s="26"/>
+      <c r="L34" s="26"/>
+      <c r="M34" s="28"/>
+      <c r="N34" s="28"/>
+      <c r="O34" s="26"/>
+      <c r="P34" s="26"/>
+      <c r="Q34" s="28"/>
+      <c r="R34" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="S34" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="T34" s="26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="28"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="26"/>
+      <c r="G35" s="26"/>
+      <c r="H35" s="26"/>
+      <c r="I35" s="28"/>
+      <c r="J35" s="26"/>
+      <c r="K35" s="26"/>
+      <c r="L35" s="26"/>
+      <c r="M35" s="28"/>
+      <c r="N35" s="28"/>
+      <c r="O35" s="26"/>
+      <c r="P35" s="26"/>
+      <c r="Q35" s="28"/>
+      <c r="R35" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="S35" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="T35" s="26">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="28"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="26"/>
+      <c r="G36" s="26"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="28"/>
+      <c r="J36" s="26"/>
+      <c r="K36" s="26"/>
+      <c r="L36" s="26"/>
+      <c r="M36" s="28"/>
+      <c r="N36" s="28"/>
+      <c r="O36" s="26"/>
+      <c r="P36" s="26"/>
+      <c r="Q36" s="28"/>
+      <c r="R36" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="S36" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="T36" s="26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="26"/>
+      <c r="B37" s="27"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="26"/>
+      <c r="F37" s="26"/>
+      <c r="G37" s="26"/>
+      <c r="H37" s="26"/>
+      <c r="I37" s="28"/>
+      <c r="J37" s="26"/>
+      <c r="K37" s="26"/>
+      <c r="L37" s="26"/>
+      <c r="M37" s="28"/>
+      <c r="N37" s="28"/>
+      <c r="O37" s="26"/>
+      <c r="P37" s="26"/>
+      <c r="Q37" s="28"/>
+      <c r="R37" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="S37" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="T37" s="26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="28"/>
+      <c r="B38" s="28"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="28"/>
+      <c r="F38" s="28"/>
+      <c r="G38" s="28"/>
+      <c r="H38" s="28"/>
+      <c r="I38" s="28"/>
+      <c r="J38" s="28"/>
+      <c r="K38" s="28"/>
+      <c r="L38" s="28"/>
+      <c r="M38" s="28"/>
+      <c r="N38" s="28"/>
+      <c r="O38" s="26"/>
+      <c r="P38" s="26"/>
+      <c r="Q38" s="28"/>
+      <c r="R38" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="S38" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="T38" s="26">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
3NF - Abiem Mahmud
</commit_message>
<xml_diff>
--- a/Normalisasi_SalesDB_Abiem Mahmud.xlsx
+++ b/Normalisasi_SalesDB_Abiem Mahmud.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arjia\magang\Latihan-database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80CCB380-77BB-4E7E-9502-67D861BF0B1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6E824DD-ADDD-4C8B-8348-D02A5A86AC61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Petunjuk" sheetId="1" r:id="rId1"/>
@@ -119,12 +119,50 @@
         </r>
       </text>
     </comment>
+    <comment ref="D27" authorId="0" shapeId="0" xr:uid="{FB36E27C-F19F-4C92-8FC9-EAA2035E896F}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Nilai tertulis di faktur asli (data sumber). Nilai ini dipertahankan sampai 3NF, lalu di sheet 4_3NF dibuktikan bahwa nilainya bisa dihitung ulang dari Qty × Harga.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Trainer</author>
+  </authors>
+  <commentList>
+    <comment ref="D13" authorId="0" shapeId="0" xr:uid="{27C0F997-7610-4966-9AC5-C72D21DF045A}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Nilai tertulis di faktur asli (data sumber). Nilai ini dipertahankan sampai 3NF, lalu di sheet 4_3NF dibuktikan bahwa nilainya bisa dihitung ulang dari Qty × Harga.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="157">
   <si>
     <t>Latihan Normalisasi SalesDB — dari data faktur (UNF) sampai 3NF</t>
   </si>
@@ -604,12 +642,6 @@
     <t>kode kategori (PK)</t>
   </si>
   <si>
-    <t>no faktur (FK)</t>
-  </si>
-  <si>
-    <t>kode produk (FK)</t>
-  </si>
-  <si>
     <t>pelanggan</t>
   </si>
   <si>
@@ -626,6 +658,15 @@
   </si>
   <si>
     <t>detail faktur</t>
+  </si>
+  <si>
+    <t>no faktur (PK, FK)</t>
+  </si>
+  <si>
+    <t>kode produk (PK,FK)</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
@@ -784,7 +825,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -811,17 +852,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -842,13 +879,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1601,46 +1638,46 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="19" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="96.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="18" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="69" x14ac:dyDescent="0.3">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="18" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="18" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="18" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="18" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="18" t="s">
         <v>106</v>
       </c>
     </row>
@@ -2259,7 +2296,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:T38"/>
+  <dimension ref="A1:U38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2306,7 +2343,7 @@
         <v>92</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>93</v>
@@ -2317,7 +2354,7 @@
         <v>94</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -2571,7 +2608,7 @@
         <v>1050000</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
         <v>68</v>
       </c>
@@ -2612,7 +2649,7 @@
         <v>346000</v>
       </c>
     </row>
-    <row r="18" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
         <v>68</v>
       </c>
@@ -2653,7 +2690,7 @@
         <v>346000</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
         <v>75</v>
       </c>
@@ -2694,7 +2731,7 @@
         <v>548000</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A20" s="12" t="s">
         <v>75</v>
       </c>
@@ -2735,7 +2772,7 @@
         <v>548000</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A21" s="12" t="s">
         <v>75</v>
       </c>
@@ -2776,7 +2813,7 @@
         <v>548000</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A22" s="12" t="s">
         <v>82</v>
       </c>
@@ -2817,7 +2854,7 @@
         <v>4450000</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:21" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
         <v>82</v>
       </c>
@@ -2858,527 +2895,538 @@
         <v>4450000</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>139</v>
       </c>
-      <c r="E25" s="21" t="s">
+      <c r="F25" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="K25" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="P25" t="s">
         <v>150</v>
       </c>
-      <c r="J25" s="21" t="s">
-        <v>151</v>
-      </c>
-      <c r="O25" t="s">
-        <v>152</v>
-      </c>
-      <c r="R25" t="s">
+      <c r="S25" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" s="23" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>129</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>138</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>156</v>
+      </c>
+      <c r="F26" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="G26" s="20" t="s">
+        <v>130</v>
+      </c>
+      <c r="H26" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="I26" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="J26" s="22"/>
+      <c r="K26" s="20" t="s">
+        <v>142</v>
+      </c>
+      <c r="L26" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="M26" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="N26" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="O26" s="22"/>
+      <c r="P26" s="20" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q26" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="R26" s="30"/>
+      <c r="S26" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="T26" s="20" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="26" spans="1:20" s="25" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="22" t="s">
-        <v>137</v>
-      </c>
-      <c r="B26" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="C26" s="22" t="s">
-        <v>138</v>
-      </c>
-      <c r="D26" s="24"/>
-      <c r="E26" s="22" t="s">
-        <v>141</v>
-      </c>
-      <c r="F26" s="22" t="s">
-        <v>130</v>
-      </c>
-      <c r="G26" s="22" t="s">
-        <v>131</v>
-      </c>
-      <c r="H26" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="I26" s="24"/>
-      <c r="J26" s="22" t="s">
-        <v>142</v>
-      </c>
-      <c r="K26" s="22" t="s">
-        <v>133</v>
-      </c>
-      <c r="L26" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="M26" s="22" t="s">
-        <v>146</v>
-      </c>
-      <c r="N26" s="24"/>
-      <c r="O26" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="P26" s="22" t="s">
-        <v>135</v>
-      </c>
-      <c r="Q26" s="32"/>
-      <c r="R26" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="S26" s="22" t="s">
-        <v>149</v>
-      </c>
-      <c r="T26" s="22" t="s">
+      <c r="U26" s="20" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="27" spans="1:20" s="30" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="26" t="s">
+    <row r="27" spans="1:21" s="28" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="B27" s="27">
+      <c r="B27" s="25">
         <v>46266</v>
       </c>
-      <c r="C27" s="26" t="s">
+      <c r="C27" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="D27" s="28"/>
-      <c r="E27" s="26" t="s">
+      <c r="D27" s="14">
+        <v>2150000</v>
+      </c>
+      <c r="F27" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="F27" s="26" t="s">
+      <c r="G27" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="G27" s="26" t="s">
+      <c r="H27" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="H27" s="26" t="s">
+      <c r="I27" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="I27" s="28"/>
-      <c r="J27" s="26" t="s">
+      <c r="J27" s="26"/>
+      <c r="K27" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="K27" s="26" t="s">
+      <c r="L27" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="L27" s="26" t="s">
+      <c r="M27" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="M27" s="29" t="s">
+      <c r="N27" s="27" t="s">
         <v>143</v>
       </c>
-      <c r="N27" s="28"/>
-      <c r="O27" s="26" t="s">
+      <c r="O27" s="26"/>
+      <c r="P27" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="P27" s="26" t="s">
+      <c r="Q27" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="Q27" s="28"/>
-      <c r="R27" s="26" t="s">
+      <c r="R27" s="26"/>
+      <c r="S27" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="S27" s="26" t="s">
+      <c r="T27" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="T27" s="26">
+      <c r="U27" s="24">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:20" s="30" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A28" s="26" t="s">
+    <row r="28" spans="1:21" s="28" customFormat="1" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="B28" s="27">
+      <c r="B28" s="25">
         <v>46275</v>
       </c>
-      <c r="C28" s="26" t="s">
+      <c r="C28" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="D28" s="28"/>
-      <c r="E28" s="26" t="s">
+      <c r="D28" s="14">
+        <v>900000</v>
+      </c>
+      <c r="F28" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="F28" s="26" t="s">
+      <c r="G28" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="G28" s="26" t="s">
+      <c r="H28" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="H28" s="26" t="s">
+      <c r="I28" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="I28" s="28"/>
-      <c r="J28" s="26" t="s">
+      <c r="J28" s="26"/>
+      <c r="K28" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="K28" s="26" t="s">
+      <c r="L28" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="L28" s="26">
+      <c r="M28" s="24">
         <v>150</v>
       </c>
-      <c r="M28" s="29" t="s">
+      <c r="N28" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="N28" s="28"/>
-      <c r="O28" s="26" t="s">
+      <c r="O28" s="26"/>
+      <c r="P28" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="P28" s="26" t="s">
+      <c r="Q28" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="Q28" s="28"/>
-      <c r="R28" s="26" t="s">
+      <c r="R28" s="26"/>
+      <c r="S28" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="S28" s="26" t="s">
+      <c r="T28" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="T28" s="26">
+      <c r="U28" s="24">
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:20" s="30" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="26" t="s">
+    <row r="29" spans="1:21" s="28" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="27">
+      <c r="B29" s="25">
         <v>46277</v>
       </c>
-      <c r="C29" s="26" t="s">
+      <c r="C29" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="D29" s="28"/>
-      <c r="E29" s="26" t="s">
+      <c r="D29" s="14">
+        <v>1050000</v>
+      </c>
+      <c r="F29" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F29" s="26" t="s">
+      <c r="G29" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="G29" s="26" t="s">
+      <c r="H29" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="H29" s="26" t="s">
+      <c r="I29" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="I29" s="28"/>
-      <c r="J29" s="26" t="s">
+      <c r="J29" s="26"/>
+      <c r="K29" s="24" t="s">
         <v>118</v>
       </c>
-      <c r="K29" s="26" t="s">
+      <c r="L29" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="L29" s="26">
+      <c r="M29" s="24">
         <v>750</v>
       </c>
-      <c r="M29" s="31" t="s">
+      <c r="N29" s="29" t="s">
         <v>144</v>
       </c>
-      <c r="N29" s="28"/>
-      <c r="O29" s="26" t="s">
+      <c r="O29" s="26"/>
+      <c r="P29" s="24" t="s">
         <v>124</v>
       </c>
-      <c r="P29" s="26" t="s">
+      <c r="Q29" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="Q29" s="28"/>
-      <c r="R29" s="26" t="s">
+      <c r="R29" s="26"/>
+      <c r="S29" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="S29" s="26" t="s">
+      <c r="T29" s="24" t="s">
         <v>118</v>
       </c>
-      <c r="T29" s="26">
+      <c r="U29" s="24">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="26" t="s">
+    <row r="30" spans="1:21" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="B30" s="27">
+      <c r="B30" s="25">
         <v>46280</v>
       </c>
-      <c r="C30" s="26" t="s">
+      <c r="C30" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="D30" s="28"/>
-      <c r="E30" s="28"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="28"/>
-      <c r="I30" s="28"/>
-      <c r="J30" s="26" t="s">
+      <c r="D30" s="14">
+        <v>346000</v>
+      </c>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="K30" s="26" t="s">
+      <c r="L30" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="L30" s="26" t="s">
+      <c r="M30" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="M30" s="31" t="s">
+      <c r="N30" s="29" t="s">
         <v>143</v>
       </c>
-      <c r="N30" s="28"/>
-      <c r="O30" s="28"/>
-      <c r="P30" s="28"/>
-      <c r="Q30" s="28"/>
-      <c r="R30" s="26" t="s">
+      <c r="O30" s="26"/>
+      <c r="P30" s="26"/>
+      <c r="Q30" s="26"/>
+      <c r="R30" s="26"/>
+      <c r="S30" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="S30" s="26" t="s">
+      <c r="T30" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="T30" s="26">
+      <c r="U30" s="24">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="26" t="s">
+    <row r="31" spans="1:21" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="B31" s="27">
+      <c r="B31" s="25">
         <v>46283</v>
       </c>
-      <c r="C31" s="26" t="s">
+      <c r="C31" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="D31" s="28"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="26" t="s">
+      <c r="D31" s="14">
+        <v>548000</v>
+      </c>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="24"/>
+      <c r="J31" s="26"/>
+      <c r="K31" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="K31" s="26" t="s">
+      <c r="L31" s="24" t="s">
         <v>122</v>
       </c>
-      <c r="L31" s="26">
+      <c r="M31" s="24">
         <v>25</v>
       </c>
-      <c r="M31" s="31" t="s">
+      <c r="N31" s="29" t="s">
         <v>145</v>
       </c>
-      <c r="N31" s="28"/>
       <c r="O31" s="26"/>
-      <c r="P31" s="26"/>
-      <c r="Q31" s="28"/>
-      <c r="R31" s="26" t="s">
+      <c r="P31" s="24"/>
+      <c r="Q31" s="24"/>
+      <c r="R31" s="26"/>
+      <c r="S31" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="S31" s="26" t="s">
+      <c r="T31" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="T31" s="26" t="s">
+      <c r="U31" s="24" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="32" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="26" t="s">
+    <row r="32" spans="1:21" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B32" s="27">
+      <c r="B32" s="25">
         <v>46285</v>
       </c>
-      <c r="C32" s="26" t="s">
+      <c r="C32" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="D32" s="28"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="26" t="s">
+      <c r="D32" s="14">
+        <v>4450000</v>
+      </c>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="24"/>
+      <c r="J32" s="26"/>
+      <c r="K32" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="K32" s="26" t="s">
+      <c r="L32" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="L32" s="26">
+      <c r="M32" s="24">
         <v>48</v>
       </c>
-      <c r="M32" s="31" t="s">
+      <c r="N32" s="29" t="s">
         <v>145</v>
       </c>
-      <c r="N32" s="28"/>
       <c r="O32" s="26"/>
-      <c r="P32" s="26"/>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="26" t="s">
+      <c r="P32" s="24"/>
+      <c r="Q32" s="24"/>
+      <c r="R32" s="26"/>
+      <c r="S32" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="S32" s="26" t="s">
+      <c r="T32" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="T32" s="26">
+      <c r="U32" s="24">
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="D33" s="28"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="28"/>
+    <row r="33" spans="1:21" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="24"/>
       <c r="J33" s="26"/>
-      <c r="K33" s="26"/>
-      <c r="L33" s="26"/>
-      <c r="M33" s="28"/>
-      <c r="N33" s="28"/>
-      <c r="O33" s="28"/>
-      <c r="P33" s="28"/>
-      <c r="Q33" s="28"/>
-      <c r="R33" s="26" t="s">
+      <c r="K33" s="24"/>
+      <c r="L33" s="24"/>
+      <c r="M33" s="24"/>
+      <c r="N33" s="26"/>
+      <c r="O33" s="26"/>
+      <c r="P33" s="26"/>
+      <c r="Q33" s="26"/>
+      <c r="R33" s="26"/>
+      <c r="S33" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="S33" s="26" t="s">
+      <c r="T33" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="T33" s="26">
+      <c r="U33" s="24">
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="26"/>
-      <c r="B34" s="27"/>
-      <c r="C34" s="26"/>
-      <c r="D34" s="28"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="28"/>
+    <row r="34" spans="1:21" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="24"/>
+      <c r="B34" s="25"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="14"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="24"/>
       <c r="J34" s="26"/>
-      <c r="K34" s="26"/>
-      <c r="L34" s="26"/>
-      <c r="M34" s="28"/>
-      <c r="N34" s="28"/>
+      <c r="K34" s="24"/>
+      <c r="L34" s="24"/>
+      <c r="M34" s="24"/>
+      <c r="N34" s="26"/>
       <c r="O34" s="26"/>
-      <c r="P34" s="26"/>
-      <c r="Q34" s="28"/>
-      <c r="R34" s="26" t="s">
+      <c r="P34" s="24"/>
+      <c r="Q34" s="24"/>
+      <c r="R34" s="26"/>
+      <c r="S34" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="S34" s="26" t="s">
+      <c r="T34" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="T34" s="26">
+      <c r="U34" s="24">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="28"/>
-      <c r="B35" s="28"/>
-      <c r="C35" s="28"/>
-      <c r="D35" s="28"/>
-      <c r="E35" s="26"/>
-      <c r="F35" s="26"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="26"/>
-      <c r="I35" s="28"/>
+    <row r="35" spans="1:21" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="26"/>
+      <c r="B35" s="26"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="14"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="24"/>
       <c r="J35" s="26"/>
-      <c r="K35" s="26"/>
-      <c r="L35" s="26"/>
-      <c r="M35" s="28"/>
-      <c r="N35" s="28"/>
+      <c r="K35" s="24"/>
+      <c r="L35" s="24"/>
+      <c r="M35" s="24"/>
+      <c r="N35" s="26"/>
       <c r="O35" s="26"/>
-      <c r="P35" s="26"/>
-      <c r="Q35" s="28"/>
-      <c r="R35" s="26" t="s">
+      <c r="P35" s="24"/>
+      <c r="Q35" s="24"/>
+      <c r="R35" s="26"/>
+      <c r="S35" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="S35" s="26" t="s">
+      <c r="T35" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="T35" s="26">
+      <c r="U35" s="24">
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="28"/>
-      <c r="B36" s="28"/>
-      <c r="C36" s="28"/>
-      <c r="D36" s="28"/>
-      <c r="E36" s="26"/>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="28"/>
+    <row r="36" spans="1:21" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="26"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="26"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="24"/>
+      <c r="I36" s="24"/>
       <c r="J36" s="26"/>
-      <c r="K36" s="26"/>
-      <c r="L36" s="26"/>
-      <c r="M36" s="28"/>
-      <c r="N36" s="28"/>
+      <c r="K36" s="24"/>
+      <c r="L36" s="24"/>
+      <c r="M36" s="24"/>
+      <c r="N36" s="26"/>
       <c r="O36" s="26"/>
-      <c r="P36" s="26"/>
-      <c r="Q36" s="28"/>
-      <c r="R36" s="26" t="s">
+      <c r="P36" s="24"/>
+      <c r="Q36" s="24"/>
+      <c r="R36" s="26"/>
+      <c r="S36" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="S36" s="26" t="s">
+      <c r="T36" s="24" t="s">
         <v>126</v>
       </c>
-      <c r="T36" s="26">
+      <c r="U36" s="24">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="26"/>
-      <c r="B37" s="27"/>
-      <c r="C37" s="26"/>
-      <c r="D37" s="28"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="26"/>
-      <c r="G37" s="26"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="28"/>
+    <row r="37" spans="1:21" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="24"/>
+      <c r="B37" s="25"/>
+      <c r="C37" s="24"/>
+      <c r="D37" s="14"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="24"/>
+      <c r="H37" s="24"/>
+      <c r="I37" s="24"/>
       <c r="J37" s="26"/>
-      <c r="K37" s="26"/>
-      <c r="L37" s="26"/>
-      <c r="M37" s="28"/>
-      <c r="N37" s="28"/>
+      <c r="K37" s="24"/>
+      <c r="L37" s="24"/>
+      <c r="M37" s="24"/>
+      <c r="N37" s="26"/>
       <c r="O37" s="26"/>
-      <c r="P37" s="26"/>
-      <c r="Q37" s="28"/>
-      <c r="R37" s="26" t="s">
+      <c r="P37" s="24"/>
+      <c r="Q37" s="24"/>
+      <c r="R37" s="26"/>
+      <c r="S37" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="S37" s="26" t="s">
+      <c r="T37" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="T37" s="26">
+      <c r="U37" s="24">
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="28"/>
-      <c r="B38" s="28"/>
-      <c r="C38" s="28"/>
-      <c r="D38" s="28"/>
-      <c r="E38" s="28"/>
-      <c r="F38" s="28"/>
-      <c r="G38" s="28"/>
-      <c r="H38" s="28"/>
-      <c r="I38" s="28"/>
-      <c r="J38" s="28"/>
-      <c r="K38" s="28"/>
-      <c r="L38" s="28"/>
-      <c r="M38" s="28"/>
-      <c r="N38" s="28"/>
+    <row r="38" spans="1:21" s="28" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="26"/>
+      <c r="B38" s="26"/>
+      <c r="C38" s="26"/>
+      <c r="F38" s="26"/>
+      <c r="G38" s="26"/>
+      <c r="H38" s="26"/>
+      <c r="I38" s="26"/>
+      <c r="J38" s="26"/>
+      <c r="K38" s="26"/>
+      <c r="L38" s="26"/>
+      <c r="M38" s="26"/>
+      <c r="N38" s="26"/>
       <c r="O38" s="26"/>
-      <c r="P38" s="26"/>
-      <c r="Q38" s="28"/>
-      <c r="R38" s="26" t="s">
+      <c r="P38" s="24"/>
+      <c r="Q38" s="24"/>
+      <c r="R38" s="26"/>
+      <c r="S38" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="S38" s="26" t="s">
+      <c r="T38" s="24" t="s">
         <v>118</v>
       </c>
-      <c r="T38" s="26">
+      <c r="U38" s="24">
         <v>1</v>
       </c>
     </row>
@@ -3389,68 +3437,627 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:C11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:U24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="21" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="16"/>
+      <c r="B6" s="16" t="s">
+        <v>136</v>
+      </c>
       <c r="C6" s="17" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="16"/>
+      <c r="B7" s="16" t="s">
+        <v>151</v>
+      </c>
       <c r="C7" s="17" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="16"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B8" s="16" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="18"/>
+    <row r="11" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
+        <v>139</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="K11" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="P11" t="s">
+        <v>150</v>
+      </c>
+      <c r="S11" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>129</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>138</v>
+      </c>
+      <c r="D12" s="21" t="s">
+        <v>156</v>
+      </c>
+      <c r="E12" s="23"/>
+      <c r="F12" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="G12" s="20" t="s">
+        <v>130</v>
+      </c>
+      <c r="H12" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="I12" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="J12" s="22"/>
+      <c r="K12" s="20" t="s">
+        <v>142</v>
+      </c>
+      <c r="L12" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="M12" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="N12" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="O12" s="22"/>
+      <c r="P12" s="20" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q12" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="R12" s="30"/>
+      <c r="S12" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="T12" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="U12" s="20" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="25">
+        <v>46266</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="14">
+        <v>2150000</v>
+      </c>
+      <c r="E13" s="28"/>
+      <c r="F13" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="H13" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="I13" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="J13" s="26"/>
+      <c r="K13" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="L13" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="M13" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="N13" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="O13" s="26"/>
+      <c r="P13" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q13" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="R13" s="26"/>
+      <c r="S13" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="T13" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="U13" s="24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="25">
+        <v>46275</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="14">
+        <v>900000</v>
+      </c>
+      <c r="E14" s="28"/>
+      <c r="F14" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="G14" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="H14" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="I14" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="J14" s="26"/>
+      <c r="K14" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="L14" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="M14" s="24">
+        <v>150</v>
+      </c>
+      <c r="N14" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="O14" s="26"/>
+      <c r="P14" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q14" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="R14" s="26"/>
+      <c r="S14" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="T14" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="U14" s="24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B15" s="25">
+        <v>46277</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="14">
+        <v>1050000</v>
+      </c>
+      <c r="E15" s="28"/>
+      <c r="F15" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="G15" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="I15" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="J15" s="26"/>
+      <c r="K15" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="L15" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="M15" s="24">
+        <v>750</v>
+      </c>
+      <c r="N15" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="O15" s="26"/>
+      <c r="P15" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q15" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="R15" s="26"/>
+      <c r="S15" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="T15" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="U15" s="24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="B16" s="25">
+        <v>46280</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="14">
+        <v>346000</v>
+      </c>
+      <c r="E16" s="28"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="26"/>
+      <c r="J16" s="26"/>
+      <c r="K16" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="L16" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="M16" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="N16" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="O16" s="26"/>
+      <c r="P16" s="26"/>
+      <c r="Q16" s="26"/>
+      <c r="R16" s="26"/>
+      <c r="S16" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="T16" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="U16" s="24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A17" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="25">
+        <v>46283</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="14">
+        <v>548000</v>
+      </c>
+      <c r="E17" s="28"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="24"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="L17" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="M17" s="24">
+        <v>25</v>
+      </c>
+      <c r="N17" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="O17" s="26"/>
+      <c r="P17" s="24"/>
+      <c r="Q17" s="24"/>
+      <c r="R17" s="26"/>
+      <c r="S17" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="T17" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="U17" s="24" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" s="25">
+        <v>46285</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="14">
+        <v>4450000</v>
+      </c>
+      <c r="E18" s="28"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="26"/>
+      <c r="K18" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="L18" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="M18" s="24">
+        <v>48</v>
+      </c>
+      <c r="N18" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="O18" s="26"/>
+      <c r="P18" s="24"/>
+      <c r="Q18" s="24"/>
+      <c r="R18" s="26"/>
+      <c r="S18" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="T18" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="U18" s="24">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="24"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="26"/>
+      <c r="K19" s="24"/>
+      <c r="L19" s="24"/>
+      <c r="M19" s="24"/>
+      <c r="N19" s="26"/>
+      <c r="O19" s="26"/>
+      <c r="P19" s="26"/>
+      <c r="Q19" s="26"/>
+      <c r="R19" s="26"/>
+      <c r="S19" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="T19" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="U19" s="24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A20" s="24"/>
+      <c r="B20" s="25"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="24"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="24"/>
+      <c r="L20" s="24"/>
+      <c r="M20" s="24"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="26"/>
+      <c r="P20" s="24"/>
+      <c r="Q20" s="24"/>
+      <c r="R20" s="26"/>
+      <c r="S20" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="T20" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="U20" s="24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A21" s="26"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="26"/>
+      <c r="K21" s="24"/>
+      <c r="L21" s="24"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="26"/>
+      <c r="O21" s="26"/>
+      <c r="P21" s="24"/>
+      <c r="Q21" s="24"/>
+      <c r="R21" s="26"/>
+      <c r="S21" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="T21" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="U21" s="24">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A22" s="26"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="24"/>
+      <c r="J22" s="26"/>
+      <c r="K22" s="24"/>
+      <c r="L22" s="24"/>
+      <c r="M22" s="24"/>
+      <c r="N22" s="26"/>
+      <c r="O22" s="26"/>
+      <c r="P22" s="24"/>
+      <c r="Q22" s="24"/>
+      <c r="R22" s="26"/>
+      <c r="S22" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="T22" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="U22" s="24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A23" s="24"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="24"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="24"/>
+      <c r="L23" s="24"/>
+      <c r="M23" s="24"/>
+      <c r="N23" s="26"/>
+      <c r="O23" s="26"/>
+      <c r="P23" s="24"/>
+      <c r="Q23" s="24"/>
+      <c r="R23" s="26"/>
+      <c r="S23" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="T23" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="U23" s="24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A24" s="26"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="26"/>
+      <c r="K24" s="26"/>
+      <c r="L24" s="26"/>
+      <c r="M24" s="26"/>
+      <c r="N24" s="26"/>
+      <c r="O24" s="26"/>
+      <c r="P24" s="24"/>
+      <c r="Q24" s="24"/>
+      <c r="R24" s="26"/>
+      <c r="S24" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="T24" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="U24" s="24">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Latihan 2.3 dan 2.4
</commit_message>
<xml_diff>
--- a/Normalisasi_SalesDB_Abiem Mahmud.xlsx
+++ b/Normalisasi_SalesDB_Abiem Mahmud.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arjia\magang\Latihan-database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAE27ACD-B73B-497C-A155-F24E3776CAFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719E0FD9-0264-4F92-8C73-436A6CD02EFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,18 @@
     <sheet name="ERD" sheetId="6" r:id="rId6"/>
     <sheet name="SCRIPT" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -140,7 +151,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="279">
   <si>
     <t>Latihan Normalisasi SalesDB — dari data faktur (UNF) sampai 3NF</t>
   </si>
@@ -6927,6 +6938,2423 @@
       </rPr>
       <t>);</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>CONSTRAINT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> CK_Product_Stock </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">CHECK </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">Stock </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>&gt;=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>),</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>INSERT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>INTO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> dbo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Category</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>OUTPUT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> inserted</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>CategoryId</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> inserted</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Name</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">VALUES </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'Batu'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>),</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'Makanan'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>),</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'Note'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>);</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>DELETE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>FROM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> dbo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Category</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>OUTPUT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> deleted</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>as</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> DeletedCategory</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>WHERE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> CategoryId </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <t>-- SEED ULANG AUTO INCREMENT</t>
+  </si>
+  <si>
+    <r>
+      <t>DBCC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> CHECKIDENT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'dbo.Category'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> RESEED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>UPDATE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> dbo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF00FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Product</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> UnitPrice </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> UnitPrice </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 1.10</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>OUTPUT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> deleted</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">UnitPrice </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>as</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> OldPrice</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> inserted</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">UnitPrice </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>as</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> NewPrice</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>WHERE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> ProductId </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> UnitPrice </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 1850000</t>
+    </r>
+  </si>
+  <si>
+    <t>-- 1. email memiliki constraint not null</t>
+  </si>
+  <si>
+    <r>
+      <t>INSERT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>INTO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> dbo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Customer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> City</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>VALUES</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>N'Dewi Lestari'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>N'Jakarta'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>);</t>
+    </r>
+  </si>
+  <si>
+    <t>-- 2. Update harga Headset</t>
+  </si>
+  <si>
+    <r>
+      <t>SET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> UnitPrice </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 375000</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>WHERE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> ProductId </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <t>-- 3. Update stok produk</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>SET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> Stock </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 15 </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>WHERE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> ProductId </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF008000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">-- monitor 1; </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">        </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>SET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> Stock </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 40 </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>WHERE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> ProductId </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF008000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">-- headset 4; </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>SET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> Stock </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 200</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>WHERE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> ProductId </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF008000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">-- Buku 5; </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>SET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> Stock </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 150 </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>WHERE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> ProductId </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF008000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">-- Pulpen 6; </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>SET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> Stock </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 60 </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>WHERE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> ProductId </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF008000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">-- Mouse 2; </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>SET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> Stock </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 25 </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>WHERE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> ProductId </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF008000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>-- Keyboard 3</t>
+    </r>
+  </si>
+  <si>
+    <t>-- 1. qty = 0</t>
+  </si>
+  <si>
+    <r>
+      <t>UPDATE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> dbo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>InvoiceDetail</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> Qty </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 0</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>WHERE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> InvoiceId </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>N'2C3024F3-8C96-40C6-B103-188018415D50'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <t>-- 2. invalid customerid</t>
+  </si>
+  <si>
+    <r>
+      <t>UPDATE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> dbo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Invoice</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> CustomerId </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> 99</t>
+    </r>
+  </si>
+  <si>
+    <t>-- 3. stock &lt; 0</t>
+  </si>
+  <si>
+    <r>
+      <t>SET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> Stock </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>5</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>BEGIN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>TRAN</t>
+    </r>
+  </si>
+  <si>
+    <t>-- 4. user baru tanpa email</t>
+  </si>
+  <si>
+    <r>
+      <t>INSERT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>INTO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> dbo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Customer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Email</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> City</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>VALUES</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>N'Eka Husna'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>NULL,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>N'Surabaya'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>);</t>
+    </r>
+  </si>
+  <si>
+    <t>-- 5. user dengan email yang sama</t>
+  </si>
+  <si>
+    <r>
+      <t>INSERT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>INTO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> dbo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Customer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>Name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> Email</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> City</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>VALUES</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>N'Tri Julian'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'budi@mail.com'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'Salatiga'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Cascadia Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>);</t>
+    </r>
+  </si>
+  <si>
+    <t>ROLLBACK</t>
+  </si>
+  <si>
+    <t>L2.3</t>
+  </si>
+  <si>
+    <t>L2.4</t>
   </si>
 </sst>
 </file>
@@ -7121,7 +9549,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -7197,6 +9625,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -10410,440 +12844,830 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{497E9FC6-F950-443E-9FBB-5EA153D29D0C}">
-  <dimension ref="A1:A93"/>
+  <dimension ref="A1:A179"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
-        <v>157</v>
-      </c>
+      <c r="A1" s="31"/>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="31" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="31" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28"/>
-    </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="28"/>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="32" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="31" t="s">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="31" t="s">
         <v>160</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="33" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="33" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="33" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="33" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="33" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" s="33" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" s="34" t="s">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" s="34" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" s="28"/>
-    </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" s="31" t="s">
+      <c r="A13" s="28"/>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" s="31" t="s">
         <v>167</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" s="33" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="33" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="33" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="33" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="33" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="34" t="s">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="34" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" s="28"/>
-    </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" s="31" t="s">
+      <c r="A20" s="28"/>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" s="31" t="s">
         <v>172</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" s="33" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="33" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="33" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="33" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="33" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="33" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" s="33" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" s="34" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" s="33" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" s="34" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A28" s="28"/>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A29" s="31" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30" s="28"/>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" s="31" t="s">
         <v>178</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A30" s="33" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A31" s="33" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" s="33" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="33" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" s="33" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" s="33" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" s="34" t="s">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" s="34" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A35" s="28"/>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A36" s="31" t="s">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37" s="28"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" s="31" t="s">
         <v>183</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A37" s="33" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A38" s="33" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" s="33" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" s="33" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" s="33" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" s="33" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A43" s="33" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A44" s="33" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A43" s="34" t="s">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A45" s="34" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A44" s="31" t="s">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A46" s="31" t="s">
         <v>158</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A45" s="28"/>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A46" s="32" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" s="28"/>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A48" s="31" t="s">
+      <c r="A48" s="32" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="28"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" s="31" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="31" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" s="28"/>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" s="31" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" s="28"/>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53" s="31" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" s="31" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" s="28"/>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" s="31" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55" s="28"/>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" s="31" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A55" s="31" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A56" s="28"/>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" s="31" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A58" s="31" t="s">
-        <v>196</v>
-      </c>
+      <c r="A58" s="28"/>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" s="31" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60" s="31" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A61" s="31" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A60" s="28"/>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A61" s="32" t="s">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A62" s="28"/>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A63" s="32" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A62" s="31" t="s">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A64" s="31" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A63" s="31" t="s">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A65" s="31" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A64" s="28"/>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A65" s="32" t="s">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A66" s="28"/>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A67" s="32" t="s">
         <v>201</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A66" s="31" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A67" s="31" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" s="31" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" s="31" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A70" s="28"/>
+      <c r="A70" s="31" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71" s="31" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A72" s="28"/>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A73" s="31" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A72" s="31" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A73" s="28"/>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" s="31" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A75" s="31" t="s">
-        <v>209</v>
-      </c>
+      <c r="A75" s="28"/>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" s="31" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" s="31" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A79" s="31" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A80" s="31" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A81" s="28"/>
+      <c r="A81" s="31" t="s">
+        <v>213</v>
+      </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A82" s="31" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A83" s="31" t="s">
-        <v>216</v>
-      </c>
+      <c r="A83" s="28"/>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A84" s="31" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A85" s="31" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A86" s="28"/>
+      <c r="A86" s="31" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A87" s="31" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A88" s="31" t="s">
-        <v>220</v>
-      </c>
+      <c r="A88" s="28"/>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A89" s="31" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A90" s="31" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A91" s="31" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A92" s="31" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A93" s="31" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A94" s="31" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A95" s="31" t="s">
         <v>225</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A96" s="28"/>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A97" s="28"/>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A98" s="31" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A99" s="31" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A100" s="31" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A101" s="28"/>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A102" s="31" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A103" s="31" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A104" s="31" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A105" s="28"/>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A106" s="32" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A107" s="31" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A108" s="28"/>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A109" s="35" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A110" s="31" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A111" s="31" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A112" s="31" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A113" s="28"/>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A114" s="35" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A115" s="31" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A116" s="31" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A117" s="31" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A118" s="28"/>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A119" s="36" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A120" s="32" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A121" s="31" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A122" s="31" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A123" s="28"/>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A124" s="32" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A125" s="35" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A126" s="31" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A127" s="31" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A128" s="28"/>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A129" s="32" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A130" s="35" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A131" s="33" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A132" s="31" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A133" s="33" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A134" s="35" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A135" s="33" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A136" s="31" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A137" s="28"/>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A138" s="35" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A139" s="33" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A140" s="31" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A141" s="28"/>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A142" s="35" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A143" s="33" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A144" s="31" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A145" s="28"/>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A146" s="35" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A147" s="33" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A148" s="31" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A149" s="28"/>
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A150" s="35" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A151" s="33" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A152" s="31" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A153" s="28"/>
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A154" s="32" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A155" s="32" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A156" s="35" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A157" s="31" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A158" s="31" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A159" s="28"/>
+    </row>
+    <row r="160" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A160" s="32" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A161" s="35" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A162" s="31" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="163" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A163" s="31" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A164" s="28"/>
+    </row>
+    <row r="165" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A165" s="32" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="166" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A166" s="35" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A167" s="31" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="168" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A168" s="31" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A169" s="28"/>
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A170" s="28"/>
+    </row>
+    <row r="171" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A171" s="31" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A172" s="32" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="173" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A173" s="31" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A174" s="31" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="175" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A175" s="28"/>
+    </row>
+    <row r="176" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A176" s="32" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A177" s="31" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A178" s="31" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A179" s="31" t="s">
+        <v>276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>